<commit_message>
chore(deps): clear remaining npm audit findings (34 → 0)
- xlsx (no patched npm release): gishub-jp scripts now read Excel with
  geopbf's own readXLSXRows (new, sheet_to_json header:1 equivalent);
  root devDep removed. readXLSX/readXLSXRows no longer mix furigana
  (<rPh>) into cell text; fixture + tests cover it.
- repomix removed (unused): devDeps in www/geopbf and summary scripts.
- adm-zip ^0.6.1 (gishub-jp, ortho-japan, sdk/japan).
- maplibre-gl devDep ^6.15.0 in geopbf (tests only); example page -> 6.11.2.
- overrides: fflate ^0.8.3 under @loaders.gl/compression; argparse ^2 /
  image-size ^2 under texture-compressor (its Node CLI is never run).

Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JpFB68khqzP61t4JnB7jd3
</commit_message>
<xml_diff>
--- a/tests/fixtures/table/book.xlsx
+++ b/tests/fixtures/table/book.xlsx
@@ -27,6 +27,10 @@
   </si>
   <si>
     <t>東京</t>
+    <rPh sb="0" eb="2">
+      <t>トウキョウ</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
   </si>
   <si>
     <t>大阪</t>

</xml_diff>